<commit_message>
TICVAI r3: the mirrors for CHG-R3-001 (derive-mirrors: the AWS LLD, the AWS workbook, the HLD/LLD pack and build-hld-lld.py in the six repos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/repos/ticvai-ai/project-bible/handoff/hld-lld/TICVAI - Azure Cloud Specs & Cost.xlsx
+++ b/ticvai/repos/ticvai-ai/project-bible/handoff/hld-lld/TICVAI - Azure Cloud Specs & Cost.xlsx
@@ -3143,7 +3143,7 @@
     <row r="43" ht="32" customHeight="1">
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>AI hosting (Chinmay, 4 October, CHG-R11-001): we host the embedding model (BGE-M3), its reranker, Presidio and the Arabic NER, together with the ticvai-ai pods, on one AI GPU node pool (NV6ads A10 v5, $473.77 a month a node; one node without HA, two with HA, one per zone); never an LLM, which stays with the providers (Core42 Compass, OpenAI UAE, BYOK). The 2 x D8s v5 AI CPU pool ($700) is gone: $8,047.50 became $8,295.04 with HA, $5,553.50 became $5,327.27 without. Defender for Containers is not re-priced for the GPU nodes' vCores (6 a node against the D8s v5's 8, so slightly lower). On AWS (me-central-1) the node is a g6.2xlarge-class instance (one L4, 8 vCPU), price and regional availability to confirm.</t>
+          <t>AI hosting (Chinmay, 4 October, CHG-R11-001): we host the embedding model (BGE-M3), its reranker, Presidio and the Arabic NER, together with the ticvai-ai pods, on one AI GPU node pool (NV6ads A10 v5, $473.77 a month a node; one node without HA, two with HA, one per zone); never an LLM, which stays with the providers (Core42 Compass, OpenAI UAE, BYOK). The 2 x D8s v5 AI CPU pool ($700) is gone: $8,047.50 became $8,295.04 with HA, $5,553.50 became $5,327.27 without. Defender for Containers is not re-priced for the GPU nodes' vCores (6 a node against the D8s v5's 8, so slightly lower). On AWS (me-central-1) the node is a g6.2xlarge (one L4 with 24 GB, 8 vCPU), $1.20043 an hour, $876.31 a month, offered in the region (AWS Price List API, 4 October; CHG-R3-001): the AWS workbook beside this one.</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>NV6ads A10 v5 (6 vCPU, 55 GB, 1/6 A10 with 4 GB), Linux, tainted, one node per zone. Carries the floors: real-time 2, interactive 1, batch 0 (about 1 vCPU a pod), Presidio on the CPU, and on the GPU at fp16 BGE-M3 (about 1.1 GB), its reranker (about 1.1 GB) and the Arabic NER (about 0.3 GB); a large cell's third real-time replica fits. No AI CPU pool and no Presidio pool. Sizing to confirm by the Sprint 2 benchmark; step up to NV12ads A10 v5 ($947.54) on CPU saturation or GPU memory pressure. AWS me-central-1: a g6.2xlarge-class node, price to confirm</t>
+          <t>NV6ads A10 v5 (6 vCPU, 55 GB, 1/6 A10 with 4 GB), Linux, tainted, one node per zone. Carries the floors: real-time 2, interactive 1, batch 0 (about 1 vCPU a pod), Presidio on the CPU, and on the GPU at fp16 BGE-M3 (about 1.1 GB), its reranker (about 1.1 GB) and the Arabic NER (about 0.3 GB); a large cell's third real-time replica fits. No AI CPU pool and no Presidio pool. Sizing to confirm by the Sprint 2 benchmark; step up to NV12ads A10 v5 ($947.54) on CPU saturation or GPU memory pressure. AWS me-central-1: g6.2xlarge ($876.31 a node; the AWS workbook, CHG-R3-001)</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
@@ -5130,7 +5130,7 @@
     <row r="44" ht="32" customHeight="1">
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>AI hosting (Chinmay, 4 October, CHG-R11-001): we host the embedding model (BGE-M3), its reranker, Presidio and the Arabic NER, together with the ticvai-ai pods, on one AI GPU node pool (NV6ads A10 v5, $473.77 a month a node; one node without HA, two with HA, one per zone); never an LLM, which stays with the providers (Core42 Compass, OpenAI UAE, BYOK). The 2 x D8s v5 AI CPU pool ($700) is gone: $8,047.50 became $8,295.04 with HA, $5,553.50 became $5,327.27 without. Defender for Containers is not re-priced for the GPU nodes' vCores (6 a node against the D8s v5's 8, so slightly lower). On AWS (me-central-1) the node is a g6.2xlarge-class instance (one L4, 8 vCPU), price and regional availability to confirm.</t>
+          <t>AI hosting (Chinmay, 4 October, CHG-R11-001): we host the embedding model (BGE-M3), its reranker, Presidio and the Arabic NER, together with the ticvai-ai pods, on one AI GPU node pool (NV6ads A10 v5, $473.77 a month a node; one node without HA, two with HA, one per zone); never an LLM, which stays with the providers (Core42 Compass, OpenAI UAE, BYOK). The 2 x D8s v5 AI CPU pool ($700) is gone: $8,047.50 became $8,295.04 with HA, $5,553.50 became $5,327.27 without. Defender for Containers is not re-priced for the GPU nodes' vCores (6 a node against the D8s v5's 8, so slightly lower). On AWS (me-central-1) the node is a g6.2xlarge (one L4 with 24 GB, 8 vCPU), $1.20043 an hour, $876.31 a month, offered in the region (AWS Price List API, 4 October; CHG-R3-001): the AWS workbook beside this one.</t>
         </is>
       </c>
     </row>

</xml_diff>